<commit_message>
Auto update schedule HTML
</commit_message>
<xml_diff>
--- a/newsletter.xlsx
+++ b/newsletter.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1546,95 +1546,95 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
+          <t>10:00～12:30</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>懐かしい盆踊りの会</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>懐かしい盆踊りのボランティア会の打ち合わせ・練習</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
           <t>14:00～16:30</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>NPO法人でんでん虫の会</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>おしゃべり会</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="n"/>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n"/>
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>10:00～12:20</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>からだケア</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>からだケア</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>10月29日（木）</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>18:30～20:30</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>一般社団法人アイ・オー・イー（IOE）</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>くまもとNPOカレッジ2026</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="n"/>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>10:00～12:00</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>特定非営利活動法人　教育支援プロジェクト・マスターズ熊本</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>トークの会</t>
-        </is>
-      </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>会</t>
+          <t>イ</t>
         </is>
       </c>
     </row>
@@ -1642,163 +1642,163 @@
       <c r="A50" s="10" t="n"/>
       <c r="B50" s="6" t="inlineStr">
         <is>
+          <t>10:00～12:00</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>特定非営利活動法人　教育支援プロジェクト・マスターズ熊本</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>トークの会</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n"/>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
           <t>13:10～15:20</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>熊本「新老人の会」</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>スポーツ吹矢</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="n"/>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="n"/>
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>18:30～20:30</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>熊本フォークダンスクラブ</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>フォークダンス練習会</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>10月30日（金）</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>13:00～17:30</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>囲碁普及会</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>囲碁の研究と対局</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="10" t="n"/>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>9:30～12:30</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>シニアクラブうらら</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>シニアいきいきサロン</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>イ・会</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="9" t="n"/>
-      <c r="B54" s="6" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="9" t="n"/>
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>13:20～17:10</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>楽しい健康吹き矢</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>吹矢を楽しむ</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>10月31日（土）</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>10:00～11:30</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>パレアひばりの会</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>フリートーキング</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="n"/>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>14:00～15:00</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>英会話サークルGreenGables</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>英会話サロン</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -1811,140 +1811,140 @@
       <c r="A57" s="10" t="n"/>
       <c r="B57" s="6" t="inlineStr">
         <is>
+          <t>14:00～15:00</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>英会話サークルGreenGables</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>英会話サロン</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
           <t>10:00～12:30</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>特定非営利活動法人 教育支援プロジェクトマスターズ熊本</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>親と子の成長を応援　親子多肉寄せ植えとリメイク鉢セミナー</t>
         </is>
       </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="n"/>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="n"/>
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>14:00～17:00</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>熊本生と死を考える会</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D59" s="7" t="inlineStr">
         <is>
           <t>熊本生と死を考える会</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>11月1日（日）</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>13:40～16:30</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr">
         <is>
           <t>ラジオ英語の会</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>英語を楽しもう</t>
         </is>
       </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="n"/>
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>14:00～16:30</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>ブレーメンの音楽隊</t>
         </is>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>音楽を楽しむ</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>11月2日（月）</t>
         </is>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>10:00～11:50</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>ヨガ健康クラブ</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>ヨガ入門</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="10" t="n"/>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>12:00～15:00</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>フラ・オ・レアレア</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>フラダンスレッスン</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -1957,17 +1957,17 @@
       <c r="A63" s="10" t="n"/>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>18:30～20:30</t>
+          <t>12:00～15:00</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>マイカ</t>
+          <t>フラ・オ・レアレア</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>フォークダンス</t>
+          <t>フラダンスレッスン</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -1980,22 +1980,22 @@
       <c r="A64" s="10" t="n"/>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>10:00～11:50</t>
+          <t>18:30～20:30</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>さわやかボランティアーズ４班</t>
+          <t>マイカ</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>さわやかボランティアーズ４班打合せ</t>
+          <t>フォークダンス</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>会</t>
+          <t>イ</t>
         </is>
       </c>
     </row>
@@ -2003,90 +2003,90 @@
       <c r="A65" s="10" t="n"/>
       <c r="B65" s="6" t="inlineStr">
         <is>
+          <t>10:00～11:50</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>さわやかボランティアーズ４班</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>さわやかボランティアーズ４班打合せ</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
           <t>14:00～15:30</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>ピエロン教室</t>
         </is>
       </c>
-      <c r="D65" s="7" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>マジックの練習</t>
         </is>
       </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="9" t="n"/>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="n"/>
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>17:20～20:30</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>楽しい健康吹き矢</t>
         </is>
       </c>
-      <c r="D66" s="7" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>吹矢を楽しむ</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>11月3日（火）</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>12:30～17:30</t>
         </is>
       </c>
-      <c r="C67" s="7" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>囲碁普及会</t>
         </is>
       </c>
-      <c r="D67" s="7" t="inlineStr">
+      <c r="D68" s="7" t="inlineStr">
         <is>
           <t>囲碁の対局・初心者の指導と研究</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="10" t="n"/>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>18:30～20:30</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>マイカ</t>
-        </is>
-      </c>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>フォークダンス</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -2099,236 +2099,236 @@
       <c r="A69" s="10" t="n"/>
       <c r="B69" s="6" t="inlineStr">
         <is>
+          <t>18:30～20:30</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>マイカ</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>フォークダンス</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="n"/>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
           <t>9:30～11:30</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>楽しいオリガミ</t>
         </is>
       </c>
-      <c r="D69" s="7" t="inlineStr">
+      <c r="D70" s="7" t="inlineStr">
         <is>
           <t>折紙製作勉強会</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="9" t="n"/>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n"/>
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>13:00～15:00</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>NPO法人傾聴ネットキーステーション</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D71" s="7" t="inlineStr">
         <is>
           <t>27期傾聴ボランティア養成講座(1回目)</t>
         </is>
       </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>11月4日（水）</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>14:00～16:30</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr">
         <is>
           <t>NPO法人でんでん虫の会</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>おしゃべり会</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="10" t="n"/>
-      <c r="B72" s="6" t="inlineStr">
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="n"/>
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>10:00～12:00</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr">
         <is>
           <t>多胎サークル　ダブルハッピー</t>
         </is>
       </c>
-      <c r="D72" s="7" t="inlineStr">
+      <c r="D73" s="7" t="inlineStr">
         <is>
           <t>多胎サークル　ダブルハッピー</t>
         </is>
       </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="n"/>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="n"/>
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>13:10～15:50</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C74" s="7" t="inlineStr">
         <is>
           <t>楽画喜の会</t>
         </is>
       </c>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="D74" s="7" t="inlineStr">
         <is>
           <t>絵画制作活動</t>
         </is>
       </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>11月5日（木）</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>12:30～14:30</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>懐かしい盆踊りの会</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
+      <c r="D75" s="7" t="inlineStr">
         <is>
           <t>懐かしい盆踊りのボランティア会の打合せ、練習</t>
         </is>
       </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="10" t="n"/>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>10:00～17:00</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C76" s="7" t="inlineStr">
         <is>
           <t>スマイリー健＆アロハ・スターハワイアンズ</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D76" s="7" t="inlineStr">
         <is>
           <t>ウクレレを楽しもう♪</t>
         </is>
       </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="9" t="n"/>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="n"/>
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>18:30～20:30</t>
         </is>
       </c>
-      <c r="C76" s="7" t="inlineStr">
+      <c r="C77" s="7" t="inlineStr">
         <is>
           <t>熊本フォークダンスクラブ</t>
         </is>
       </c>
-      <c r="D76" s="7" t="inlineStr">
+      <c r="D77" s="7" t="inlineStr">
         <is>
           <t>フォークダンス練習会</t>
         </is>
       </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>11月6日（金）</t>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>9:30～12:30</t>
         </is>
       </c>
-      <c r="C77" s="7" t="inlineStr">
+      <c r="C78" s="7" t="inlineStr">
         <is>
           <t>シニアクラブうらら</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>シニアいきいきサロン</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="10" t="n"/>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>13:30～15:30</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>NPO法人熊本わくわく体操ボランティア協会</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>いつでも・だれでも健康体操</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -2341,240 +2341,240 @@
       <c r="A79" s="10" t="n"/>
       <c r="B79" s="6" t="inlineStr">
         <is>
+          <t>13:30～15:30</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>NPO法人熊本わくわく体操ボランティア協会</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>いつでも・だれでも健康体操</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n"/>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
           <t>10:00～11:30</t>
         </is>
       </c>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>熊本健康マージャン協会</t>
         </is>
       </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>マージャン協会の座談会</t>
         </is>
       </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="9" t="n"/>
-      <c r="B80" s="6" t="inlineStr">
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="n"/>
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>14:30～17:30</t>
         </is>
       </c>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C81" s="7" t="inlineStr">
         <is>
           <t>スマイリー健＆アロハ・スターハワイアンズ</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D81" s="7" t="inlineStr">
         <is>
           <t>♪ハワイアン・懐メロ演奏会♪</t>
         </is>
       </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr">
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
         <is>
           <t>11月7日（土）</t>
         </is>
       </c>
-      <c r="B81" s="6" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>13:30～16:30</t>
         </is>
       </c>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>東教養囲碁研究会</t>
         </is>
       </c>
-      <c r="D81" s="7" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
         <is>
           <t>囲碁による人間形成・修練</t>
         </is>
       </c>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="10" t="n"/>
-      <c r="B82" s="6" t="inlineStr">
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n"/>
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>10:00～13:00</t>
         </is>
       </c>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="C83" s="7" t="inlineStr">
         <is>
           <t>特定非営利活動法人教育支援プロジェクトマスターズ熊本</t>
         </is>
       </c>
-      <c r="D82" s="7" t="inlineStr">
+      <c r="D83" s="7" t="inlineStr">
         <is>
           <t>教育支援プロジェクトマスターズ熊本20周年記念事業</t>
         </is>
       </c>
-      <c r="E82" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="9" t="n"/>
-      <c r="B83" s="6" t="inlineStr">
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="n"/>
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>13:30～16:30</t>
         </is>
       </c>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr">
         <is>
           <t>傾聴ボランティアくまもと</t>
         </is>
       </c>
-      <c r="D83" s="7" t="inlineStr">
+      <c r="D84" s="7" t="inlineStr">
         <is>
           <t>傾聴定例会</t>
         </is>
       </c>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="5" t="inlineStr">
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>11月8日（日）</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>10:00～12:00</t>
         </is>
       </c>
-      <c r="C84" s="7" t="inlineStr">
+      <c r="C85" s="7" t="inlineStr">
         <is>
           <t>さわやか南京玉すだれを楽しむ会</t>
         </is>
       </c>
-      <c r="D84" s="7" t="inlineStr">
+      <c r="D85" s="7" t="inlineStr">
         <is>
           <t>南京玉すだれの練習</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="9" t="n"/>
-      <c r="B85" s="6" t="inlineStr">
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="n"/>
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>10:00～11:10</t>
         </is>
       </c>
-      <c r="C85" s="7" t="inlineStr">
+      <c r="C86" s="7" t="inlineStr">
         <is>
           <t>口からの健康づくり 歯っぴーかむカム</t>
         </is>
       </c>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="D86" s="7" t="inlineStr">
         <is>
           <t>ベロタッチ生活養生・食養生</t>
         </is>
       </c>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>11月9日（月）</t>
-        </is>
-      </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>18:30～20:30</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>マイカ</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>フォークダンス</t>
-        </is>
-      </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>イ</t>
+          <t>会</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
+          <t>11月9日（月）</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>18:30～20:30</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>マイカ</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>フォークダンス</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
           <t>11月10日（火）</t>
         </is>
       </c>
-      <c r="B87" s="6" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>9:30～12:00</t>
         </is>
       </c>
-      <c r="C87" s="7" t="inlineStr">
+      <c r="C88" s="7" t="inlineStr">
         <is>
           <t>はなの風</t>
         </is>
       </c>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="D88" s="7" t="inlineStr">
         <is>
           <t>はなの風（水彩画教室）</t>
-        </is>
-      </c>
-      <c r="E87" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="10" t="n"/>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>12:30～17:30</t>
-        </is>
-      </c>
-      <c r="C88" s="7" t="inlineStr">
-        <is>
-          <t>囲碁普及会</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>囲碁の対局・初心者の指導と研究</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -2587,17 +2587,17 @@
       <c r="A89" s="10" t="n"/>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>19:00～20:30</t>
+          <t>12:30～17:30</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>熊本市キャンプ協会</t>
+          <t>囲碁普及会</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>定例会</t>
+          <t>囲碁の対局・初心者の指導と研究</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -2610,22 +2610,22 @@
       <c r="A90" s="10" t="n"/>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>10:00～12:00</t>
+          <t>19:00～20:30</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>太極拳を楽しもう会</t>
+          <t>熊本市キャンプ協会</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>健康太極拳</t>
+          <t>定例会</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>会</t>
+          <t>イ</t>
         </is>
       </c>
     </row>
@@ -2633,90 +2633,90 @@
       <c r="A91" s="10" t="n"/>
       <c r="B91" s="6" t="inlineStr">
         <is>
+          <t>10:00～12:00</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>太極拳を楽しもう会</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>健康太極拳</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n"/>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
           <t>13:00～15:00</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>NPO法人傾聴ネットキーステーション</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>27期傾聴ボランティア養成講座(2回目)</t>
         </is>
       </c>
-      <c r="E91" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="9" t="n"/>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="n"/>
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>19:30～20:30</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>笑顔のたまて箱</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
         <is>
           <t>人形劇の練習及び打合せ</t>
         </is>
       </c>
-      <c r="E92" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="5" t="inlineStr">
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t>11月11日（水）</t>
         </is>
       </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>9:40～11:30</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>KKA高齢者健康友の会</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>みんな笑顔で楽しく健康体操</t>
-        </is>
-      </c>
-      <c r="E93" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="10" t="n"/>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>10:00～12:00</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr">
-        <is>
-          <t>（一社）熊本県助産師会</t>
-        </is>
-      </c>
-      <c r="D94" s="7" t="inlineStr">
-        <is>
-          <t>ママ＆ベビー教室</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
@@ -2729,90 +2729,90 @@
       <c r="A95" s="10" t="n"/>
       <c r="B95" s="6" t="inlineStr">
         <is>
+          <t>10:00～12:00</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>（一社）熊本県助産師会</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>ママ＆ベビー教室</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n"/>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
           <t>14:00～16:30</t>
         </is>
       </c>
-      <c r="C95" s="7" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>NPO法人でんでん虫の会</t>
         </is>
       </c>
-      <c r="D95" s="7" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>おしゃべり会</t>
         </is>
       </c>
-      <c r="E95" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="9" t="n"/>
-      <c r="B96" s="6" t="inlineStr">
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="n"/>
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>13:30～17:30</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>「アミーゴ」</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
         <is>
           <t>「アミーゴ」バンド活動</t>
         </is>
       </c>
-      <c r="E96" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="5" t="inlineStr">
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
         <is>
           <t>11月13日（金）</t>
         </is>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B98" s="6" t="inlineStr">
         <is>
           <t>13:00～17:30</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C98" s="7" t="inlineStr">
         <is>
           <t>囲碁普及会</t>
         </is>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="D98" s="7" t="inlineStr">
         <is>
           <t>囲碁の研究と対局</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="10" t="n"/>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>18:30～20:30</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>一般社団法人アイ・オー・イー（IOE）</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>くまもとNPOカレッジ2026</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -2825,22 +2825,22 @@
       <c r="A99" s="10" t="n"/>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>9:30～12:30</t>
+          <t>18:30～20:30</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>シニアクラブうらら</t>
+          <t>一般社団法人アイ・オー・イー（IOE）</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>シニアいきいきサロン</t>
+          <t>くまもとNPOカレッジ2026</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>会</t>
+          <t>イ</t>
         </is>
       </c>
     </row>
@@ -2848,90 +2848,90 @@
       <c r="A100" s="10" t="n"/>
       <c r="B100" s="6" t="inlineStr">
         <is>
+          <t>9:30～12:30</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>シニアクラブうらら</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>シニアいきいきサロン</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="n"/>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
           <t>12:30～17:00</t>
         </is>
       </c>
-      <c r="C100" s="7" t="inlineStr">
+      <c r="C101" s="7" t="inlineStr">
         <is>
           <t>AA九州・沖縄地域熊本地区</t>
         </is>
       </c>
-      <c r="D100" s="7" t="inlineStr">
+      <c r="D101" s="7" t="inlineStr">
         <is>
           <t>AA九州・沖縄地域 矯正・保護施設フォーラムin熊本</t>
         </is>
       </c>
-      <c r="E100" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="n"/>
+      <c r="B102" s="6" t="inlineStr">
         <is>
           <t>18:30～20:30</t>
         </is>
       </c>
-      <c r="C101" s="7" t="inlineStr">
+      <c r="C102" s="7" t="inlineStr">
         <is>
           <t>熊本フォークダンスクラブ</t>
         </is>
       </c>
-      <c r="D101" s="7" t="inlineStr">
+      <c r="D102" s="7" t="inlineStr">
         <is>
           <t>フォークダンス練習会</t>
         </is>
       </c>
-      <c r="E101" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="5" t="inlineStr">
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
         <is>
           <t>11月14日（土）</t>
         </is>
       </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="B103" s="6" t="inlineStr">
         <is>
           <t>9:00～11:50</t>
         </is>
       </c>
-      <c r="C102" s="7" t="inlineStr">
+      <c r="C103" s="7" t="inlineStr">
         <is>
           <t>熊本さわやかハイヤ俱楽部</t>
         </is>
       </c>
-      <c r="D102" s="7" t="inlineStr">
+      <c r="D103" s="7" t="inlineStr">
         <is>
           <t>熊本の郷土芸能「牛深ハイヤ踊り」の練習</t>
-        </is>
-      </c>
-      <c r="E102" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="10" t="n"/>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>13:30～16:30</t>
-        </is>
-      </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>東教養囲碁研究会</t>
-        </is>
-      </c>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t>囲碁による人間形成・修練</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -2944,90 +2944,90 @@
       <c r="A104" s="10" t="n"/>
       <c r="B104" s="6" t="inlineStr">
         <is>
+          <t>13:30～16:30</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>東教養囲碁研究会</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>囲碁による人間形成・修練</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="n"/>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
           <t>9:00～11:50</t>
         </is>
       </c>
-      <c r="C104" s="7" t="inlineStr">
+      <c r="C105" s="7" t="inlineStr">
         <is>
           <t>熊本史談会</t>
         </is>
       </c>
-      <c r="D104" s="7" t="inlineStr">
+      <c r="D105" s="7" t="inlineStr">
         <is>
           <t>熊本歴史の勉強会</t>
         </is>
       </c>
-      <c r="E104" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="9" t="n"/>
-      <c r="B105" s="6" t="inlineStr">
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="n"/>
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>13:30～16:30</t>
         </is>
       </c>
-      <c r="C105" s="7" t="inlineStr">
+      <c r="C106" s="7" t="inlineStr">
         <is>
           <t>登校拒否・不登校に学ぶフレンズネットワークくまもと</t>
         </is>
       </c>
-      <c r="D105" s="7" t="inlineStr">
+      <c r="D106" s="7" t="inlineStr">
         <is>
           <t>フレンズ親の会</t>
         </is>
       </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
         <is>
           <t>11月15日（日）</t>
         </is>
       </c>
-      <c r="B106" s="6" t="inlineStr">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>9:00～12:30</t>
         </is>
       </c>
-      <c r="C106" s="7" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr">
         <is>
           <t>特定非営利活動法人 教育支援プロジェクトマスターズ熊本</t>
         </is>
       </c>
-      <c r="D106" s="7" t="inlineStr">
+      <c r="D107" s="7" t="inlineStr">
         <is>
           <t>親と子の体験　クリスマスプレート作り(陶磁器)</t>
-        </is>
-      </c>
-      <c r="E106" s="8" t="inlineStr">
-        <is>
-          <t>イ</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="10" t="n"/>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>13:40～16:30</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>ラジオ英語の会</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>英語を楽しもう</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -3040,43 +3040,66 @@
       <c r="A108" s="10" t="n"/>
       <c r="B108" s="6" t="inlineStr">
         <is>
+          <t>13:40～16:30</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="inlineStr">
+        <is>
+          <t>ラジオ英語の会</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr">
+        <is>
+          <t>英語を楽しもう</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>イ</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="n"/>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
           <t>11:00～12:00</t>
         </is>
       </c>
-      <c r="C108" s="7" t="inlineStr">
+      <c r="C109" s="7" t="inlineStr">
         <is>
           <t>くまもと琵琶楽普及会</t>
         </is>
       </c>
-      <c r="D108" s="7" t="inlineStr">
+      <c r="D109" s="7" t="inlineStr">
         <is>
           <t>ワークショップ 琵琶の音色を楽しむ</t>
         </is>
       </c>
-      <c r="E108" s="8" t="inlineStr">
-        <is>
-          <t>会</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="9" t="n"/>
-      <c r="B109" s="6" t="inlineStr">
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>会</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="n"/>
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>15:00～17:30</t>
         </is>
       </c>
-      <c r="C109" s="7" t="inlineStr">
+      <c r="C110" s="7" t="inlineStr">
         <is>
           <t>「アミーゴ」</t>
         </is>
       </c>
-      <c r="D109" s="7" t="inlineStr">
+      <c r="D110" s="7" t="inlineStr">
         <is>
           <t>高齢者バンド</t>
         </is>
       </c>
-      <c r="E109" s="8" t="inlineStr">
+      <c r="E110" s="8" t="inlineStr">
         <is>
           <t>会</t>
         </is>
@@ -3084,35 +3107,35 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A67:A70"/>
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="A84:A85"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="A60:A61"/>
+    <mergeCell ref="A107:A110"/>
     <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A72:A74"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A81:A83"/>
-    <mergeCell ref="A97:A101"/>
-    <mergeCell ref="A61:A66"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A103:A106"/>
+    <mergeCell ref="A53:A55"/>
+    <mergeCell ref="A88:A93"/>
     <mergeCell ref="A9:A13"/>
-    <mergeCell ref="A52:A54"/>
-    <mergeCell ref="A87:A92"/>
+    <mergeCell ref="A56:A59"/>
     <mergeCell ref="A28:A32"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A85:A86"/>
     <mergeCell ref="A33:A36"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A18:A23"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A82:A84"/>
     <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A98:A102"/>
     <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A93:A96"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A77:A80"/>
-    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A75:A77"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="A46:A48"/>
     <mergeCell ref="A24:A27"/>
     <mergeCell ref="A37:A41"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="A62:A67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>